<commit_message>
Atualizacao automatica da base
</commit_message>
<xml_diff>
--- a/dados/despesas_2026_08.xlsx
+++ b/dados/despesas_2026_08.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd3092d5ed7ea8c4/Área de Trabalho/Cris/Python/Dash_Dagmar/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{C44A4EB1-4844-4325-A8A9-2218A2A8E917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{568DF74C-6A09-46F4-9739-D7DEB6FD32D8}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{C44A4EB1-4844-4325-A8A9-2218A2A8E917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8902C23-3F7F-4857-A154-7BA677ABEE44}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{825677E9-9EF4-4190-B89E-F41040B0586F}"/>
   </bookViews>
@@ -1563,13 +1563,13 @@
         <v>14</v>
       </c>
       <c r="E2" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F2" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="G2" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="H2" s="2">
         <v>875.02</v>
@@ -1607,13 +1607,13 @@
         <v>17</v>
       </c>
       <c r="E3" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F3" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="G3" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="H3" s="2">
         <v>603.54999999999995</v>
@@ -1651,13 +1651,13 @@
         <v>18</v>
       </c>
       <c r="E4" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F4" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="G4" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="H4" s="2">
         <v>33.44</v>
@@ -1695,13 +1695,13 @@
         <v>19</v>
       </c>
       <c r="E5" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F5" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="G5" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="H5" s="2">
         <v>3.77</v>
@@ -1739,13 +1739,13 @@
         <v>20</v>
       </c>
       <c r="E6" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F6" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="G6" s="1">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="H6" s="2">
         <v>19.3</v>
@@ -1783,13 +1783,13 @@
         <v>22</v>
       </c>
       <c r="E7" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F7" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G7" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H7" s="2">
         <v>1164.02</v>
@@ -1827,13 +1827,13 @@
         <v>22</v>
       </c>
       <c r="E8" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F8" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G8" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H8" s="2">
         <v>1169.6099999999999</v>
@@ -1871,13 +1871,13 @@
         <v>22</v>
       </c>
       <c r="E9" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F9" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G9" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H9" s="2">
         <v>1470.09</v>
@@ -1915,13 +1915,13 @@
         <v>22</v>
       </c>
       <c r="E10" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F10" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G10" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H10" s="2">
         <v>1999.45</v>
@@ -1959,13 +1959,13 @@
         <v>23</v>
       </c>
       <c r="E11" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F11" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G11" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H11" s="2">
         <v>2.16</v>
@@ -2003,13 +2003,13 @@
         <v>20</v>
       </c>
       <c r="E12" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F12" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G12" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H12" s="2">
         <v>4929.3</v>
@@ -2047,13 +2047,13 @@
         <v>19</v>
       </c>
       <c r="E13" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F13" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G13" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H13" s="2">
         <v>185.74</v>
@@ -2091,13 +2091,13 @@
         <v>19</v>
       </c>
       <c r="E14" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F14" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G14" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H14" s="2">
         <v>1.81</v>
@@ -2135,13 +2135,13 @@
         <v>24</v>
       </c>
       <c r="E15" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F15" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G15" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H15" s="2">
         <v>139.75</v>
@@ -2179,13 +2179,13 @@
         <v>23</v>
       </c>
       <c r="E16" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F16" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G16" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H16" s="2">
         <v>413.7</v>
@@ -2223,13 +2223,13 @@
         <v>25</v>
       </c>
       <c r="E17" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F17" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G17" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H17" s="2">
         <v>819.59</v>
@@ -2267,13 +2267,13 @@
         <v>24</v>
       </c>
       <c r="E18" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F18" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G18" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H18" s="2">
         <v>115.84</v>
@@ -2311,13 +2311,13 @@
         <v>24</v>
       </c>
       <c r="E19" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F19" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G19" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H19" s="2">
         <v>182.61</v>
@@ -2355,13 +2355,13 @@
         <v>19</v>
       </c>
       <c r="E20" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F20" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G20" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H20" s="2">
         <v>19.170000000000002</v>
@@ -2399,13 +2399,13 @@
         <v>23</v>
       </c>
       <c r="E21" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F21" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="G21" s="1">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="H21" s="2">
         <v>110.41</v>
@@ -2443,13 +2443,13 @@
         <v>19</v>
       </c>
       <c r="E22" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F22" s="1">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="G22" s="1">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="H22" s="2">
         <v>1.9</v>
@@ -2487,13 +2487,13 @@
         <v>19</v>
       </c>
       <c r="E23" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F23" s="1">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="G23" s="1">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="H23" s="2">
         <v>24.46</v>
@@ -2531,13 +2531,13 @@
         <v>22</v>
       </c>
       <c r="E24" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F24" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G24" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H24" s="2">
         <v>2196.9699999999998</v>
@@ -2575,13 +2575,13 @@
         <v>27</v>
       </c>
       <c r="E25" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F25" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G25" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H25" s="2">
         <v>1291.3800000000001</v>
@@ -2619,13 +2619,13 @@
         <v>28</v>
       </c>
       <c r="E26" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F26" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G26" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H26" s="2">
         <v>745.93</v>
@@ -2663,13 +2663,13 @@
         <v>29</v>
       </c>
       <c r="E27" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F27" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G27" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H27" s="2">
         <v>278.67</v>
@@ -2707,13 +2707,13 @@
         <v>29</v>
       </c>
       <c r="E28" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F28" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G28" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H28" s="2">
         <v>336.53</v>
@@ -2751,13 +2751,13 @@
         <v>30</v>
       </c>
       <c r="E29" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F29" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G29" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H29" s="2">
         <v>1014.74</v>
@@ -2795,13 +2795,13 @@
         <v>31</v>
       </c>
       <c r="E30" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F30" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G30" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H30" s="2">
         <v>109.14</v>
@@ -2839,13 +2839,13 @@
         <v>19</v>
       </c>
       <c r="E31" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F31" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G31" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H31" s="2">
         <v>2.52</v>
@@ -2883,13 +2883,13 @@
         <v>19</v>
       </c>
       <c r="E32" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F32" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G32" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="H32" s="2">
         <v>25.09</v>
@@ -2927,13 +2927,13 @@
         <v>32</v>
       </c>
       <c r="E33" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F33" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G33" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H33" s="2">
         <v>1349.64</v>
@@ -2971,13 +2971,13 @@
         <v>19</v>
       </c>
       <c r="E34" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F34" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G34" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H34" s="2">
         <v>2.1800000000000002</v>
@@ -3015,13 +3015,13 @@
         <v>33</v>
       </c>
       <c r="E35" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F35" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G35" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H35" s="2">
         <v>2262.59</v>
@@ -3059,13 +3059,13 @@
         <v>34</v>
       </c>
       <c r="E36" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F36" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G36" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H36" s="2">
         <v>2970.89</v>
@@ -3103,13 +3103,13 @@
         <v>35</v>
       </c>
       <c r="E37" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F37" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G37" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H37" s="2">
         <v>634.82000000000005</v>
@@ -3147,13 +3147,13 @@
         <v>36</v>
       </c>
       <c r="E38" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F38" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G38" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H38" s="2">
         <v>57.26</v>
@@ -3191,13 +3191,13 @@
         <v>35</v>
       </c>
       <c r="E39" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F39" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G39" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H39" s="2">
         <v>1262.67</v>
@@ -3235,13 +3235,13 @@
         <v>38</v>
       </c>
       <c r="E40" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F40" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G40" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H40" s="2">
         <v>43</v>
@@ -3279,13 +3279,13 @@
         <v>38</v>
       </c>
       <c r="E41" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F41" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G41" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H41" s="2">
         <v>77.11</v>
@@ -3323,13 +3323,13 @@
         <v>38</v>
       </c>
       <c r="E42" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F42" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G42" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H42" s="2">
         <v>29.57</v>
@@ -3367,13 +3367,13 @@
         <v>38</v>
       </c>
       <c r="E43" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F43" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G43" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H43" s="2">
         <v>44.76</v>
@@ -3411,13 +3411,13 @@
         <v>35</v>
       </c>
       <c r="E44" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F44" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G44" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H44" s="2">
         <v>524.95000000000005</v>
@@ -3455,13 +3455,13 @@
         <v>38</v>
       </c>
       <c r="E45" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F45" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G45" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H45" s="2">
         <v>61</v>
@@ -3499,13 +3499,13 @@
         <v>39</v>
       </c>
       <c r="E46" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F46" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G46" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H46" s="2">
         <v>7.7</v>
@@ -3543,13 +3543,13 @@
         <v>41</v>
       </c>
       <c r="E47" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F47" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G47" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H47" s="2">
         <v>20.8</v>
@@ -3587,13 +3587,13 @@
         <v>41</v>
       </c>
       <c r="E48" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F48" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G48" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H48" s="2">
         <v>34.6</v>
@@ -3631,13 +3631,13 @@
         <v>41</v>
       </c>
       <c r="E49" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F49" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G49" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H49" s="2">
         <v>21.51</v>
@@ -3675,13 +3675,13 @@
         <v>42</v>
       </c>
       <c r="E50" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F50" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G50" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H50" s="2">
         <v>58.71</v>
@@ -3719,13 +3719,13 @@
         <v>43</v>
       </c>
       <c r="E51" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F51" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G51" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H51" s="2">
         <v>14.17</v>
@@ -3763,13 +3763,13 @@
         <v>45</v>
       </c>
       <c r="E52" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F52" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G52" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H52" s="2">
         <v>55.86</v>
@@ -3807,13 +3807,13 @@
         <v>41</v>
       </c>
       <c r="E53" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F53" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G53" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H53" s="2">
         <v>10.050000000000001</v>
@@ -3851,13 +3851,13 @@
         <v>41</v>
       </c>
       <c r="E54" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F54" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G54" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H54" s="2">
         <v>13.15</v>
@@ -3895,13 +3895,13 @@
         <v>41</v>
       </c>
       <c r="E55" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F55" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G55" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H55" s="2">
         <v>25.15</v>
@@ -3939,13 +3939,13 @@
         <v>35</v>
       </c>
       <c r="E56" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F56" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G56" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H56" s="2">
         <v>1507.73</v>
@@ -3983,13 +3983,13 @@
         <v>35</v>
       </c>
       <c r="E57" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F57" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G57" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H57" s="2">
         <v>1005.28</v>
@@ -4027,13 +4027,13 @@
         <v>35</v>
       </c>
       <c r="E58" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F58" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G58" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H58" s="2">
         <v>835.29</v>
@@ -4071,13 +4071,13 @@
         <v>35</v>
       </c>
       <c r="E59" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F59" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G59" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H59" s="2">
         <v>1087.71</v>
@@ -4115,13 +4115,13 @@
         <v>35</v>
       </c>
       <c r="E60" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F60" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G60" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H60" s="2">
         <v>1603.15</v>
@@ -4159,13 +4159,13 @@
         <v>35</v>
       </c>
       <c r="E61" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F61" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G61" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H61" s="2">
         <v>1758.73</v>
@@ -4203,13 +4203,13 @@
         <v>35</v>
       </c>
       <c r="E62" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F62" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G62" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H62" s="2">
         <v>2101.19</v>
@@ -4247,13 +4247,13 @@
         <v>35</v>
       </c>
       <c r="E63" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F63" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G63" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H63" s="2">
         <v>1461.23</v>
@@ -4291,13 +4291,13 @@
         <v>35</v>
       </c>
       <c r="E64" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F64" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G64" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H64" s="2">
         <v>1490.13</v>
@@ -4335,13 +4335,13 @@
         <v>48</v>
       </c>
       <c r="E65" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F65" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G65" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H65" s="2">
         <v>308.5</v>
@@ -4379,13 +4379,13 @@
         <v>35</v>
       </c>
       <c r="E66" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F66" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G66" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H66" s="2">
         <v>2094.34</v>
@@ -4423,13 +4423,13 @@
         <v>35</v>
       </c>
       <c r="E67" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F67" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G67" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H67" s="2">
         <v>2173.79</v>
@@ -4467,13 +4467,13 @@
         <v>35</v>
       </c>
       <c r="E68" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F68" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G68" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H68" s="2">
         <v>1375.76</v>
@@ -4511,13 +4511,13 @@
         <v>35</v>
       </c>
       <c r="E69" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F69" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G69" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H69" s="2">
         <v>169.44</v>
@@ -4555,13 +4555,13 @@
         <v>19</v>
       </c>
       <c r="E70" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F70" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="G70" s="1">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="H70" s="2">
         <v>43.98</v>
@@ -4599,13 +4599,13 @@
         <v>41</v>
       </c>
       <c r="E71" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F71" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="G71" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="H71" s="2">
         <v>4.72</v>
@@ -4643,13 +4643,13 @@
         <v>50</v>
       </c>
       <c r="E72" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F72" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="G72" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="H72" s="2">
         <v>185.12</v>
@@ -4687,13 +4687,13 @@
         <v>51</v>
       </c>
       <c r="E73" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F73" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="G73" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="H73" s="2">
         <v>83.64</v>
@@ -4731,13 +4731,13 @@
         <v>53</v>
       </c>
       <c r="E74" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F74" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G74" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H74" s="2">
         <v>303.52</v>
@@ -4775,13 +4775,13 @@
         <v>54</v>
       </c>
       <c r="E75" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F75" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G75" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H75" s="2">
         <v>12538.23</v>
@@ -4819,13 +4819,13 @@
         <v>54</v>
       </c>
       <c r="E76" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F76" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G76" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H76" s="2">
         <v>1126.6500000000001</v>
@@ -4863,13 +4863,13 @@
         <v>27</v>
       </c>
       <c r="E77" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F77" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G77" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H77" s="2">
         <v>224.37</v>
@@ -4907,13 +4907,13 @@
         <v>56</v>
       </c>
       <c r="E78" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F78" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G78" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H78" s="2">
         <v>35504.199999999997</v>
@@ -4951,13 +4951,13 @@
         <v>58</v>
       </c>
       <c r="E79" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F79" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G79" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H79" s="2">
         <v>556.41999999999996</v>
@@ -4995,13 +4995,13 @@
         <v>30</v>
       </c>
       <c r="E80" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F80" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G80" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H80" s="2">
         <v>602.71</v>
@@ -5039,13 +5039,13 @@
         <v>19</v>
       </c>
       <c r="E81" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F81" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G81" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H81" s="2">
         <v>4.42</v>
@@ -5083,13 +5083,13 @@
         <v>59</v>
       </c>
       <c r="E82" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F82" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G82" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H82" s="2">
         <v>118.2</v>
@@ -5127,13 +5127,13 @@
         <v>36</v>
       </c>
       <c r="E83" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F83" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G83" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H83" s="2">
         <v>121.05</v>
@@ -5171,13 +5171,13 @@
         <v>36</v>
       </c>
       <c r="E84" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F84" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G84" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H84" s="2">
         <v>93.35</v>
@@ -5215,13 +5215,13 @@
         <v>20</v>
       </c>
       <c r="E85" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F85" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="G85" s="1">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="H85" s="2">
         <v>664.56</v>
@@ -5259,13 +5259,13 @@
         <v>34</v>
       </c>
       <c r="E86" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F86" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G86" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H86" s="2">
         <v>1570.48</v>
@@ -5303,13 +5303,13 @@
         <v>34</v>
       </c>
       <c r="E87" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F87" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G87" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H87" s="2">
         <v>2970.51</v>
@@ -5347,13 +5347,13 @@
         <v>34</v>
       </c>
       <c r="E88" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F88" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G88" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H88" s="2">
         <v>4863.1499999999996</v>
@@ -5391,13 +5391,13 @@
         <v>34</v>
       </c>
       <c r="E89" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F89" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G89" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H89" s="2">
         <v>499.93</v>
@@ -5435,13 +5435,13 @@
         <v>34</v>
       </c>
       <c r="E90" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F90" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G90" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H90" s="2">
         <v>1175.9100000000001</v>
@@ -5479,13 +5479,13 @@
         <v>34</v>
       </c>
       <c r="E91" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F91" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G91" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H91" s="2">
         <v>690.92</v>
@@ -5523,13 +5523,13 @@
         <v>34</v>
       </c>
       <c r="E92" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F92" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G92" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H92" s="2">
         <v>1332.36</v>
@@ -5567,13 +5567,13 @@
         <v>34</v>
       </c>
       <c r="E93" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F93" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G93" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H93" s="2">
         <v>2413.0100000000002</v>
@@ -5611,13 +5611,13 @@
         <v>34</v>
       </c>
       <c r="E94" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F94" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G94" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H94" s="2">
         <v>1917.89</v>
@@ -5655,13 +5655,13 @@
         <v>34</v>
       </c>
       <c r="E95" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F95" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G95" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H95" s="2">
         <v>1047.31</v>
@@ -5699,13 +5699,13 @@
         <v>34</v>
       </c>
       <c r="E96" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F96" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G96" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H96" s="2">
         <v>1784.39</v>
@@ -5743,13 +5743,13 @@
         <v>38</v>
       </c>
       <c r="E97" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F97" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G97" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H97" s="2">
         <v>3368.15</v>
@@ -5787,13 +5787,13 @@
         <v>34</v>
       </c>
       <c r="E98" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F98" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G98" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H98" s="2">
         <v>1380.9</v>
@@ -5831,13 +5831,13 @@
         <v>34</v>
       </c>
       <c r="E99" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F99" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G99" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H99" s="2">
         <v>788.63</v>
@@ -5875,13 +5875,13 @@
         <v>34</v>
       </c>
       <c r="E100" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F100" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G100" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H100" s="2">
         <v>744</v>
@@ -5919,13 +5919,13 @@
         <v>34</v>
       </c>
       <c r="E101" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F101" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G101" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H101" s="2">
         <v>3790.44</v>
@@ -5963,13 +5963,13 @@
         <v>19</v>
       </c>
       <c r="E102" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F102" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G102" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H102" s="2">
         <v>103</v>
@@ -6007,13 +6007,13 @@
         <v>66</v>
       </c>
       <c r="E103" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F103" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G103" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H103" s="2">
         <v>872.43</v>
@@ -6051,13 +6051,13 @@
         <v>66</v>
       </c>
       <c r="E104" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F104" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G104" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H104" s="2">
         <v>1053.45</v>
@@ -6095,13 +6095,13 @@
         <v>66</v>
       </c>
       <c r="E105" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F105" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G105" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H105" s="2">
         <v>334.46</v>
@@ -6139,13 +6139,13 @@
         <v>66</v>
       </c>
       <c r="E106" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F106" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G106" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H106" s="2">
         <v>983.55</v>
@@ -6183,13 +6183,13 @@
         <v>66</v>
       </c>
       <c r="E107" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F107" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G107" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H107" s="2">
         <v>644.46</v>
@@ -6227,13 +6227,13 @@
         <v>66</v>
       </c>
       <c r="E108" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F108" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G108" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H108" s="2">
         <v>1174.76</v>
@@ -6271,13 +6271,13 @@
         <v>66</v>
       </c>
       <c r="E109" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F109" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G109" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H109" s="2">
         <v>652.36</v>
@@ -6315,13 +6315,13 @@
         <v>66</v>
       </c>
       <c r="E110" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F110" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G110" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H110" s="2">
         <v>1483.3</v>
@@ -6359,13 +6359,13 @@
         <v>66</v>
       </c>
       <c r="E111" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F111" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G111" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H111" s="2">
         <v>514.62</v>
@@ -6403,13 +6403,13 @@
         <v>66</v>
       </c>
       <c r="E112" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F112" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G112" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H112" s="2">
         <v>702.85</v>
@@ -6447,13 +6447,13 @@
         <v>66</v>
       </c>
       <c r="E113" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F113" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G113" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H113" s="2">
         <v>1677.06</v>
@@ -6491,13 +6491,13 @@
         <v>66</v>
       </c>
       <c r="E114" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F114" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G114" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H114" s="2">
         <v>1318.8</v>
@@ -6535,13 +6535,13 @@
         <v>36</v>
       </c>
       <c r="E115" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F115" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G115" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H115" s="2">
         <v>128.44</v>
@@ -6579,13 +6579,13 @@
         <v>66</v>
       </c>
       <c r="E116" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F116" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G116" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H116" s="2">
         <v>749.3</v>
@@ -6623,13 +6623,13 @@
         <v>66</v>
       </c>
       <c r="E117" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F117" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G117" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H117" s="2">
         <v>2344.58</v>
@@ -6667,13 +6667,13 @@
         <v>68</v>
       </c>
       <c r="E118" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F118" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G118" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H118" s="2">
         <v>12.99</v>
@@ -6711,13 +6711,13 @@
         <v>66</v>
       </c>
       <c r="E119" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F119" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G119" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H119" s="2">
         <v>832.56</v>
@@ -6755,13 +6755,13 @@
         <v>19</v>
       </c>
       <c r="E120" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F120" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="G120" s="1">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="H120" s="2">
         <v>100.04</v>
@@ -6799,13 +6799,13 @@
         <v>34</v>
       </c>
       <c r="E121" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F121" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G121" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H121" s="2">
         <v>2885.99</v>
@@ -6843,13 +6843,13 @@
         <v>30</v>
       </c>
       <c r="E122" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F122" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G122" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H122" s="2">
         <v>1338.88</v>
@@ -6887,13 +6887,13 @@
         <v>33</v>
       </c>
       <c r="E123" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F123" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G123" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H123" s="2">
         <v>2334.0300000000002</v>
@@ -6931,13 +6931,13 @@
         <v>25</v>
       </c>
       <c r="E124" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F124" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G124" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H124" s="2">
         <v>336.19</v>
@@ -6975,13 +6975,13 @@
         <v>25</v>
       </c>
       <c r="E125" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F125" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G125" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H125" s="2">
         <v>20.239999999999998</v>
@@ -7019,13 +7019,13 @@
         <v>38</v>
       </c>
       <c r="E126" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F126" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G126" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H126" s="2">
         <v>676.89</v>
@@ -7063,13 +7063,13 @@
         <v>51</v>
       </c>
       <c r="E127" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F127" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G127" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H127" s="2">
         <v>54.47</v>
@@ -7107,13 +7107,13 @@
         <v>38</v>
       </c>
       <c r="E128" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F128" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G128" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H128" s="2">
         <v>1125.73</v>
@@ -7151,13 +7151,13 @@
         <v>38</v>
       </c>
       <c r="E129" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F129" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G129" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H129" s="2">
         <v>389.17</v>
@@ -7195,13 +7195,13 @@
         <v>38</v>
       </c>
       <c r="E130" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F130" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G130" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H130" s="2">
         <v>343.48</v>
@@ -7239,13 +7239,13 @@
         <v>38</v>
       </c>
       <c r="E131" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F131" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G131" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H131" s="2">
         <v>545.25</v>
@@ -7283,13 +7283,13 @@
         <v>38</v>
       </c>
       <c r="E132" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F132" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G132" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H132" s="2">
         <v>209.9</v>
@@ -7327,13 +7327,13 @@
         <v>38</v>
       </c>
       <c r="E133" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F133" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G133" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H133" s="2">
         <v>665.72</v>
@@ -7371,13 +7371,13 @@
         <v>38</v>
       </c>
       <c r="E134" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F134" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G134" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H134" s="2">
         <v>49.4</v>
@@ -7415,13 +7415,13 @@
         <v>73</v>
       </c>
       <c r="E135" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F135" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G135" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H135" s="2">
         <v>22.2</v>
@@ -7459,13 +7459,13 @@
         <v>41</v>
       </c>
       <c r="E136" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F136" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G136" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H136" s="2">
         <v>6.21</v>
@@ -7503,13 +7503,13 @@
         <v>38</v>
       </c>
       <c r="E137" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F137" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G137" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H137" s="2">
         <v>291.01</v>
@@ -7547,13 +7547,13 @@
         <v>34</v>
       </c>
       <c r="E138" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F138" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G138" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H138" s="2">
         <v>350.92</v>
@@ -7591,13 +7591,13 @@
         <v>30</v>
       </c>
       <c r="E139" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F139" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G139" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H139" s="2">
         <v>14.69</v>
@@ -7635,13 +7635,13 @@
         <v>39</v>
       </c>
       <c r="E140" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F140" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G140" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H140" s="2">
         <v>106.73</v>
@@ -7679,13 +7679,13 @@
         <v>19</v>
       </c>
       <c r="E141" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F141" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="G141" s="1">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="H141" s="2">
         <v>4.67</v>
@@ -7723,13 +7723,13 @@
         <v>33</v>
       </c>
       <c r="E142" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F142" s="1">
-        <v>46215</v>
+        <v>46246</v>
       </c>
       <c r="G142" s="1">
-        <v>46215</v>
+        <v>46246</v>
       </c>
       <c r="H142" s="2">
         <v>225.32</v>
@@ -7767,13 +7767,13 @@
         <v>25</v>
       </c>
       <c r="E143" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F143" s="1">
-        <v>46215</v>
+        <v>46246</v>
       </c>
       <c r="G143" s="1">
-        <v>46215</v>
+        <v>46246</v>
       </c>
       <c r="H143" s="2">
         <v>202.91</v>
@@ -7811,13 +7811,13 @@
         <v>38</v>
       </c>
       <c r="E144" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F144" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G144" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H144" s="2">
         <v>294.20999999999998</v>
@@ -7855,13 +7855,13 @@
         <v>66</v>
       </c>
       <c r="E145" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F145" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G145" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H145" s="2">
         <v>228.13</v>
@@ -7899,13 +7899,13 @@
         <v>19</v>
       </c>
       <c r="E146" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F146" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G146" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H146" s="2">
         <v>718.32</v>
@@ -7943,13 +7943,13 @@
         <v>19</v>
       </c>
       <c r="E147" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F147" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G147" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H147" s="2">
         <v>6.84</v>
@@ -7987,13 +7987,13 @@
         <v>74</v>
       </c>
       <c r="E148" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F148" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G148" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H148" s="2">
         <v>1073.8800000000001</v>
@@ -8031,13 +8031,13 @@
         <v>19</v>
       </c>
       <c r="E149" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F149" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G149" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H149" s="2">
         <v>5.38</v>
@@ -8075,13 +8075,13 @@
         <v>20</v>
       </c>
       <c r="E150" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F150" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G150" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H150" s="2">
         <v>4315.09</v>
@@ -8119,13 +8119,13 @@
         <v>31</v>
       </c>
       <c r="E151" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F151" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G151" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="H151" s="2">
         <v>206.04</v>
@@ -8163,13 +8163,13 @@
         <v>36</v>
       </c>
       <c r="E152" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F152" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G152" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H152" s="2">
         <v>108.95</v>
@@ -8207,13 +8207,13 @@
         <v>41</v>
       </c>
       <c r="E153" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F153" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G153" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H153" s="2">
         <v>91.1</v>
@@ -8251,13 +8251,13 @@
         <v>42</v>
       </c>
       <c r="E154" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F154" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G154" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H154" s="2">
         <v>57.53</v>
@@ -8295,13 +8295,13 @@
         <v>45</v>
       </c>
       <c r="E155" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F155" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G155" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H155" s="2">
         <v>37.01</v>
@@ -8339,13 +8339,13 @@
         <v>41</v>
       </c>
       <c r="E156" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F156" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G156" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H156" s="2">
         <v>15.22</v>
@@ -8383,13 +8383,13 @@
         <v>41</v>
       </c>
       <c r="E157" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F157" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G157" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H157" s="2">
         <v>39.79</v>
@@ -8427,13 +8427,13 @@
         <v>76</v>
       </c>
       <c r="E158" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F158" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G158" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H158" s="2">
         <v>1201.06</v>
@@ -8471,13 +8471,13 @@
         <v>77</v>
       </c>
       <c r="E159" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F159" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G159" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H159" s="2">
         <v>1999.7</v>
@@ -8515,13 +8515,13 @@
         <v>19</v>
       </c>
       <c r="E160" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F160" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G160" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H160" s="2">
         <v>3.4</v>
@@ -8559,13 +8559,13 @@
         <v>78</v>
       </c>
       <c r="E161" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F161" s="1">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="G161" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H161" s="2">
         <v>1332.33</v>
@@ -8603,13 +8603,13 @@
         <v>79</v>
       </c>
       <c r="E162" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F162" s="1">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="G162" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H162" s="2">
         <v>1757.47</v>
@@ -8647,13 +8647,13 @@
         <v>50</v>
       </c>
       <c r="E163" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F163" s="1">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="G163" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H163" s="2">
         <v>1001.3</v>
@@ -8691,13 +8691,13 @@
         <v>82</v>
       </c>
       <c r="E164" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F164" s="1">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="G164" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H164" s="2">
         <v>258.07</v>
@@ -8735,13 +8735,13 @@
         <v>77</v>
       </c>
       <c r="E165" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F165" s="1">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="G165" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H165" s="2">
         <v>530.75</v>
@@ -8779,13 +8779,13 @@
         <v>14</v>
       </c>
       <c r="E166" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F166" s="1">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="G166" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H166" s="2">
         <v>668.59</v>
@@ -8823,13 +8823,13 @@
         <v>84</v>
       </c>
       <c r="E167" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F167" s="1">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="G167" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H167" s="2">
         <v>605.74</v>
@@ -8867,13 +8867,13 @@
         <v>19</v>
       </c>
       <c r="E168" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F168" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G168" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H168" s="2">
         <v>2.94</v>
@@ -8911,13 +8911,13 @@
         <v>27</v>
       </c>
       <c r="E169" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F169" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G169" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H169" s="2">
         <v>116.55</v>
@@ -8955,13 +8955,13 @@
         <v>34</v>
       </c>
       <c r="E170" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F170" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G170" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H170" s="2">
         <v>678.47</v>
@@ -8999,13 +8999,13 @@
         <v>30</v>
       </c>
       <c r="E171" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F171" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G171" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H171" s="2">
         <v>146.13</v>
@@ -9043,13 +9043,13 @@
         <v>36</v>
       </c>
       <c r="E172" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F172" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="G172" s="1">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="H172" s="2">
         <v>110.74</v>
@@ -9087,13 +9087,13 @@
         <v>86</v>
       </c>
       <c r="E173" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F173" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G173" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H173" s="2">
         <v>26813.7</v>
@@ -9131,13 +9131,13 @@
         <v>87</v>
       </c>
       <c r="E174" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F174" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G174" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H174" s="2">
         <v>3631.68</v>
@@ -9175,13 +9175,13 @@
         <v>68</v>
       </c>
       <c r="E175" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F175" s="1">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="G175" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H175" s="2">
         <v>260.61</v>
@@ -9219,13 +9219,13 @@
         <v>41</v>
       </c>
       <c r="E176" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F176" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G176" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H176" s="2">
         <v>7.63</v>
@@ -9263,13 +9263,13 @@
         <v>90</v>
       </c>
       <c r="E177" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F177" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G177" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H177" s="2">
         <v>43</v>
@@ -9307,13 +9307,13 @@
         <v>38</v>
       </c>
       <c r="E178" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F178" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G178" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H178" s="2">
         <v>289.16000000000003</v>
@@ -9351,13 +9351,13 @@
         <v>38</v>
       </c>
       <c r="E179" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F179" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G179" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H179" s="2">
         <v>94.17</v>
@@ -9395,13 +9395,13 @@
         <v>38</v>
       </c>
       <c r="E180" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F180" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G180" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H180" s="2">
         <v>51.51</v>
@@ -9439,13 +9439,13 @@
         <v>91</v>
       </c>
       <c r="E181" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F181" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G181" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H181" s="2">
         <v>158.91</v>
@@ -9483,13 +9483,13 @@
         <v>38</v>
       </c>
       <c r="E182" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F182" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G182" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H182" s="2">
         <v>122.31</v>
@@ -9527,13 +9527,13 @@
         <v>38</v>
       </c>
       <c r="E183" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F183" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G183" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H183" s="2">
         <v>111.61</v>
@@ -9571,13 +9571,13 @@
         <v>38</v>
       </c>
       <c r="E184" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F184" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G184" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H184" s="2">
         <v>73.22</v>
@@ -9615,13 +9615,13 @@
         <v>33</v>
       </c>
       <c r="E185" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F185" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G185" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H185" s="2">
         <v>302.77999999999997</v>
@@ -9659,13 +9659,13 @@
         <v>51</v>
       </c>
       <c r="E186" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F186" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G186" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H186" s="2">
         <v>579.54999999999995</v>
@@ -9703,13 +9703,13 @@
         <v>41</v>
       </c>
       <c r="E187" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F187" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G187" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H187" s="2">
         <v>12.75</v>
@@ -9747,13 +9747,13 @@
         <v>38</v>
       </c>
       <c r="E188" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F188" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G188" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H188" s="2">
         <v>48.95</v>
@@ -9791,13 +9791,13 @@
         <v>38</v>
       </c>
       <c r="E189" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F189" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G189" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H189" s="2">
         <v>43.43</v>
@@ -9835,13 +9835,13 @@
         <v>41</v>
       </c>
       <c r="E190" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F190" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G190" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="H190" s="2">
         <v>46.63</v>
@@ -9879,13 +9879,13 @@
         <v>92</v>
       </c>
       <c r="E191" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F191" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G191" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H191" s="2">
         <v>746.6</v>
@@ -9923,13 +9923,13 @@
         <v>27</v>
       </c>
       <c r="E192" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F192" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G192" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H192" s="2">
         <v>586.22</v>
@@ -9967,13 +9967,13 @@
         <v>27</v>
       </c>
       <c r="E193" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F193" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G193" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H193" s="2">
         <v>1097.53</v>
@@ -10011,13 +10011,13 @@
         <v>29</v>
       </c>
       <c r="E194" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F194" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G194" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H194" s="2">
         <v>294.02</v>
@@ -10055,13 +10055,13 @@
         <v>22</v>
       </c>
       <c r="E195" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F195" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G195" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H195" s="2">
         <v>1830.9</v>
@@ -10099,13 +10099,13 @@
         <v>22</v>
       </c>
       <c r="E196" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F196" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G196" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H196" s="2">
         <v>1373.7</v>
@@ -10143,13 +10143,13 @@
         <v>19</v>
       </c>
       <c r="E197" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F197" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="G197" s="1">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="H197" s="2">
         <v>3.88</v>
@@ -10187,13 +10187,13 @@
         <v>41</v>
       </c>
       <c r="E198" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F198" s="1">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="G198" s="1">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="H198" s="2">
         <v>263.32</v>
@@ -10231,13 +10231,13 @@
         <v>95</v>
       </c>
       <c r="E199" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F199" s="1">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="G199" s="1">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="H199" s="2">
         <v>2989.69</v>
@@ -10275,13 +10275,13 @@
         <v>19</v>
       </c>
       <c r="E200" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F200" s="1">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="G200" s="1">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="H200" s="2">
         <v>2.4500000000000002</v>
@@ -10319,13 +10319,13 @@
         <v>38</v>
       </c>
       <c r="E201" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F201" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G201" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H201" s="2">
         <v>342.5</v>
@@ -10363,13 +10363,13 @@
         <v>38</v>
       </c>
       <c r="E202" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F202" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G202" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H202" s="2">
         <v>350.96</v>
@@ -10407,13 +10407,13 @@
         <v>38</v>
       </c>
       <c r="E203" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F203" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G203" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H203" s="2">
         <v>188.89</v>
@@ -10451,13 +10451,13 @@
         <v>38</v>
       </c>
       <c r="E204" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F204" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G204" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H204" s="2">
         <v>94.55</v>
@@ -10495,13 +10495,13 @@
         <v>38</v>
       </c>
       <c r="E205" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F205" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G205" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H205" s="2">
         <v>28.13</v>
@@ -10539,13 +10539,13 @@
         <v>18</v>
       </c>
       <c r="E206" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F206" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G206" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H206" s="2">
         <v>33.869999999999997</v>
@@ -10583,13 +10583,13 @@
         <v>25</v>
       </c>
       <c r="E207" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F207" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G207" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H207" s="2">
         <v>55.24</v>
@@ -10627,13 +10627,13 @@
         <v>36</v>
       </c>
       <c r="E208" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F208" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="G208" s="1">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="H208" s="2">
         <v>81.11</v>
@@ -10671,13 +10671,13 @@
         <v>96</v>
       </c>
       <c r="E209" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F209" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="G209" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="H209" s="2">
         <v>274.25</v>
@@ -10715,13 +10715,13 @@
         <v>51</v>
       </c>
       <c r="E210" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F210" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="G210" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="H210" s="2">
         <v>62.84</v>
@@ -10759,13 +10759,13 @@
         <v>92</v>
       </c>
       <c r="E211" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F211" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="G211" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="H211" s="2">
         <v>25415.82</v>
@@ -10803,13 +10803,13 @@
         <v>30</v>
       </c>
       <c r="E212" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F212" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="G212" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="H212" s="2">
         <v>971.57</v>
@@ -10847,13 +10847,13 @@
         <v>30</v>
       </c>
       <c r="E213" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F213" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="G213" s="1">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="H213" s="2">
         <v>1387.78</v>
@@ -10891,13 +10891,13 @@
         <v>36</v>
       </c>
       <c r="E214" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F214" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G214" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H214" s="2">
         <v>70.67</v>
@@ -10935,13 +10935,13 @@
         <v>36</v>
       </c>
       <c r="E215" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F215" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G215" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H215" s="2">
         <v>75.92</v>
@@ -10979,13 +10979,13 @@
         <v>19</v>
       </c>
       <c r="E216" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F216" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G216" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H216" s="2">
         <v>1563.08</v>
@@ -11023,13 +11023,13 @@
         <v>97</v>
       </c>
       <c r="E217" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F217" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G217" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H217" s="2">
         <v>12678.39</v>
@@ -11067,13 +11067,13 @@
         <v>97</v>
       </c>
       <c r="E218" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F218" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G218" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H218" s="2">
         <v>10767.63</v>
@@ -11111,13 +11111,13 @@
         <v>20</v>
       </c>
       <c r="E219" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F219" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G219" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H219" s="2">
         <v>2513.52</v>
@@ -11155,13 +11155,13 @@
         <v>20</v>
       </c>
       <c r="E220" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F220" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G220" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H220" s="2">
         <v>2052.75</v>
@@ -11199,13 +11199,13 @@
         <v>19</v>
       </c>
       <c r="E221" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F221" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="G221" s="1">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="H221" s="2">
         <v>1.87</v>
@@ -11243,13 +11243,13 @@
         <v>30</v>
       </c>
       <c r="E222" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F222" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="G222" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="H222" s="2">
         <v>968.32</v>
@@ -11287,13 +11287,13 @@
         <v>30</v>
       </c>
       <c r="E223" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F223" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="G223" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="H223" s="2">
         <v>61.09</v>
@@ -11331,13 +11331,13 @@
         <v>91</v>
       </c>
       <c r="E224" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F224" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="G224" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="H224" s="2">
         <v>38.5</v>
@@ -11375,13 +11375,13 @@
         <v>38</v>
       </c>
       <c r="E225" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F225" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="G225" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="H225" s="2">
         <v>238.8</v>
@@ -11419,13 +11419,13 @@
         <v>19</v>
       </c>
       <c r="E226" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F226" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="G226" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="H226" s="2">
         <v>1.5</v>
@@ -11463,13 +11463,13 @@
         <v>38</v>
       </c>
       <c r="E227" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F227" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G227" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H227" s="2">
         <v>195.71</v>
@@ -11507,13 +11507,13 @@
         <v>38</v>
       </c>
       <c r="E228" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F228" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G228" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H228" s="2">
         <v>159.44</v>
@@ -11551,13 +11551,13 @@
         <v>30</v>
       </c>
       <c r="E229" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F229" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G229" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H229" s="2">
         <v>485.35</v>
@@ -11595,13 +11595,13 @@
         <v>91</v>
       </c>
       <c r="E230" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F230" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G230" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H230" s="2">
         <v>281.79000000000002</v>
@@ -11639,13 +11639,13 @@
         <v>91</v>
       </c>
       <c r="E231" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F231" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G231" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H231" s="2">
         <v>293.73</v>
@@ -11683,13 +11683,13 @@
         <v>91</v>
       </c>
       <c r="E232" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F232" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G232" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H232" s="2">
         <v>371.53</v>
@@ -11727,13 +11727,13 @@
         <v>91</v>
       </c>
       <c r="E233" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F233" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G233" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H233" s="2">
         <v>201.21</v>
@@ -11771,13 +11771,13 @@
         <v>91</v>
       </c>
       <c r="E234" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F234" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G234" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H234" s="2">
         <v>428.04</v>
@@ -11815,13 +11815,13 @@
         <v>91</v>
       </c>
       <c r="E235" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F235" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G235" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H235" s="2">
         <v>629.23</v>
@@ -11859,13 +11859,13 @@
         <v>92</v>
       </c>
       <c r="E236" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F236" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G236" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H236" s="2">
         <v>855.13</v>
@@ -11903,13 +11903,13 @@
         <v>102</v>
       </c>
       <c r="E237" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F237" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G237" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H237" s="2">
         <v>3711.76</v>
@@ -11947,13 +11947,13 @@
         <v>104</v>
       </c>
       <c r="E238" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F238" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G238" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H238" s="2">
         <v>2315.8000000000002</v>
@@ -11991,13 +11991,13 @@
         <v>91</v>
       </c>
       <c r="E239" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F239" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G239" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H239" s="2">
         <v>4803.4799999999996</v>
@@ -12035,13 +12035,13 @@
         <v>18</v>
       </c>
       <c r="E240" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F240" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G240" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H240" s="2">
         <v>32.299999999999997</v>
@@ -12079,13 +12079,13 @@
         <v>91</v>
       </c>
       <c r="E241" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F241" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G241" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H241" s="2">
         <v>327.39</v>
@@ -12123,13 +12123,13 @@
         <v>106</v>
       </c>
       <c r="E242" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F242" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G242" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H242" s="2">
         <v>316.66000000000003</v>
@@ -12167,13 +12167,13 @@
         <v>38</v>
       </c>
       <c r="E243" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F243" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G243" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H243" s="2">
         <v>1188.95</v>
@@ -12211,13 +12211,13 @@
         <v>42</v>
       </c>
       <c r="E244" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F244" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G244" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H244" s="2">
         <v>29.79</v>
@@ -12255,13 +12255,13 @@
         <v>34</v>
       </c>
       <c r="E245" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F245" s="1">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="G245" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H245" s="2">
         <v>288.22000000000003</v>
@@ -12299,13 +12299,13 @@
         <v>107</v>
       </c>
       <c r="E246" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F246" s="1">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="G246" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H246" s="2">
         <v>8.1</v>
@@ -12343,13 +12343,13 @@
         <v>108</v>
       </c>
       <c r="E247" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F247" s="1">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="G247" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H247" s="2">
         <v>4003.85</v>
@@ -12387,13 +12387,13 @@
         <v>73</v>
       </c>
       <c r="E248" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F248" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G248" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H248" s="2">
         <v>75.48</v>
@@ -12431,13 +12431,13 @@
         <v>41</v>
       </c>
       <c r="E249" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F249" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G249" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H249" s="2">
         <v>3.29</v>
@@ -12475,13 +12475,13 @@
         <v>38</v>
       </c>
       <c r="E250" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F250" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G250" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H250" s="2">
         <v>277.97000000000003</v>
@@ -12519,13 +12519,13 @@
         <v>42</v>
       </c>
       <c r="E251" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F251" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G251" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H251" s="2">
         <v>77.84</v>
@@ -12563,13 +12563,13 @@
         <v>41</v>
       </c>
       <c r="E252" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F252" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G252" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H252" s="2">
         <v>7.61</v>
@@ -12607,13 +12607,13 @@
         <v>38</v>
       </c>
       <c r="E253" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F253" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G253" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H253" s="2">
         <v>392.73</v>
@@ -12651,13 +12651,13 @@
         <v>38</v>
       </c>
       <c r="E254" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F254" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G254" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H254" s="2">
         <v>59.38</v>
@@ -12695,13 +12695,13 @@
         <v>38</v>
       </c>
       <c r="E255" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F255" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G255" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H255" s="2">
         <v>36.67</v>
@@ -12739,13 +12739,13 @@
         <v>38</v>
       </c>
       <c r="E256" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F256" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="G256" s="1">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="H256" s="2">
         <v>31</v>
@@ -12783,13 +12783,13 @@
         <v>109</v>
       </c>
       <c r="E257" s="3">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="F257" s="1">
         <v>46247</v>
       </c>
       <c r="G257" s="1">
-        <v>46216</v>
+        <v>46247</v>
       </c>
       <c r="H257" s="2">
         <v>2525.36</v>

</xml_diff>